<commit_message>
Actualizar archivo de casos de prueba
</commit_message>
<xml_diff>
--- a/trabajofinalcasosdeprueba.xlsx
+++ b/trabajofinalcasosdeprueba.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leont\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{98C9E7DF-40B8-474B-9043-5C7D15F2405A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37576800-73FB-4DB5-ABB2-99602B6EF1D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B8935615-B3F4-41A7-891D-83988B98A047}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
   <si>
     <t>Casos Normales</t>
   </si>
@@ -173,6 +173,15 @@
   </si>
   <si>
     <t>ERROR, no cumple la edad minima de 57 años (mujer) para adquirir el derecho a la pension</t>
+  </si>
+  <si>
+    <t>Entrada</t>
+  </si>
+  <si>
+    <t>Salida</t>
+  </si>
+  <si>
+    <t>Proceso</t>
   </si>
 </sst>
 </file>
@@ -186,7 +195,7 @@
     <numFmt numFmtId="167" formatCode="0.00\%"/>
     <numFmt numFmtId="168" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,8 +214,29 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -231,8 +261,26 @@
         <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -255,11 +303,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -282,6 +339,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3642A87F-1BF7-4509-BE1A-2ECAF5D37DAF}">
-  <dimension ref="A2:O21"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.5546875" customWidth="1"/>
@@ -628,6 +700,32 @@
     <col min="15" max="15" width="86.109375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:15" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B1" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="16"/>
+      <c r="D1" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="18" t="s">
+        <v>43</v>
+      </c>
+    </row>
     <row r="2" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
@@ -671,7 +769,7 @@
       <c r="N2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="17" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1678,6 +1776,11 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:N1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>